<commit_message>
updated method agent - searching within local docs
</commit_message>
<xml_diff>
--- a/python/data/Реестр_адапт_мер.xlsx
+++ b/python/data/Реестр_адапт_мер.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nasty\OneDrive\Рабочий стол\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nasty\Desktop\climate_measures\python\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94920E40-582E-4980-B3CE-5D3C08F62254}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB94C3BB-F0FB-4131-88CA-859AAE02DE04}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8688" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="усиление адаптивной способности" sheetId="4" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="127">
   <si>
     <t>Адаптационная потребность</t>
   </si>
@@ -519,7 +519,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="0"/>
         <bgColor theme="7" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
@@ -551,7 +551,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top"/>
@@ -580,71 +580,68 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -902,20 +899,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F94"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="30.5546875" style="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.88671875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.44140625" style="27" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="63.109375" style="27" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="27"/>
-    <col min="8" max="8" width="9.109375" style="27" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="27"/>
+    <col min="1" max="1" width="30.53125" style="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.86328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.46484375" style="22" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="63.1328125" style="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.1328125" style="22"/>
+    <col min="8" max="8" width="9.1328125" style="22" customWidth="1"/>
+    <col min="9" max="16384" width="9.1328125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="27.6">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="27">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -935,25 +932,25 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="27.6">
-      <c r="A2" s="15" t="s">
+    <row r="2" spans="1:6" ht="27">
+      <c r="A2" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="23" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="27.6">
-      <c r="A3" s="15" t="s">
+    <row r="3" spans="1:6" ht="27">
+      <c r="A3" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -965,12 +962,12 @@
       <c r="D3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="41.4">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:6" ht="27">
+      <c r="A4" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -980,12 +977,12 @@
         <v>21</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="27" t="s">
+      <c r="E4" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="55.2">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:6" ht="40.5">
+      <c r="A5" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="7" t="s">
@@ -995,12 +992,12 @@
         <v>7</v>
       </c>
       <c r="D5" s="9"/>
-      <c r="E5" s="27" t="s">
+      <c r="E5" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="69">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:6" ht="67.5">
+      <c r="A6" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -1010,12 +1007,12 @@
         <v>21</v>
       </c>
       <c r="D6" s="9"/>
-      <c r="E6" s="27" t="s">
+      <c r="E6" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="27.6">
-      <c r="A7" s="15" t="s">
+    <row r="7" spans="1:6" ht="27">
+      <c r="A7" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -1025,12 +1022,12 @@
         <v>13</v>
       </c>
       <c r="D7" s="9"/>
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="41.4">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:6" ht="40.5">
+      <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="9" t="s">
@@ -1042,12 +1039,12 @@
       <c r="D8" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="55.2">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:6" ht="54">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
@@ -1059,12 +1056,12 @@
       <c r="D9" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="41.4">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:6" ht="27">
+      <c r="A10" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="9" t="s">
@@ -1076,320 +1073,320 @@
       <c r="D10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="55.2">
-      <c r="A11" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="10" t="s">
+    <row r="11" spans="1:6" ht="54">
+      <c r="A11" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="28" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="41.4">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:6" ht="40.5">
+      <c r="A12" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="27" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="28" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="41.4">
-      <c r="A13" s="26" t="s">
+    <row r="13" spans="1:6" ht="40.5">
+      <c r="A13" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="28" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="22" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="41.4">
-      <c r="A14" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="15" t="s">
+    <row r="14" spans="1:6" ht="40.5">
+      <c r="A14" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="13" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="41.4">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:6" ht="27">
+      <c r="A15" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="41.4">
-      <c r="A16" s="15" t="s">
+    <row r="16" spans="1:6" ht="40.5">
+      <c r="A16" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="15" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="9"/>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="55.2">
-      <c r="A17" s="15" t="s">
+    <row r="17" spans="1:6" ht="54">
+      <c r="A17" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="15" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="9"/>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="27.6">
-      <c r="A18" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="15" t="s">
+    <row r="18" spans="1:6" ht="27">
+      <c r="A18" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="15" t="s">
         <v>21</v>
       </c>
       <c r="D18" s="9"/>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="41.4">
-      <c r="A19" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="15" t="s">
+    <row r="19" spans="1:6" ht="40.5">
+      <c r="A19" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="15" t="s">
         <v>13</v>
       </c>
       <c r="D19" s="9"/>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="14" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="41.4">
-      <c r="A20" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="19" t="s">
+    <row r="20" spans="1:6" ht="40.5">
+      <c r="A20" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="17" t="s">
         <v>13</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="F20" s="21" t="s">
+      <c r="F20" s="18" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="41.4">
-      <c r="A21" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="22" t="s">
+    <row r="21" spans="1:6" ht="40.5">
+      <c r="A21" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="17" t="s">
         <v>13</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="55.2">
-      <c r="A22" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" s="22" t="s">
+    <row r="22" spans="1:6" ht="54">
+      <c r="A22" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="17" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E22" s="27" t="s">
+      <c r="E22" s="22" t="s">
         <v>124</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="27.6">
-      <c r="A23" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="23" t="s">
+    <row r="23" spans="1:6" ht="27">
+      <c r="A23" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="17" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="9"/>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="22" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="23" t="s">
+      <c r="A24" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="C24" s="20" t="s">
+      <c r="C24" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D24" s="9"/>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="22" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="23" t="s">
+      <c r="A25" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="17" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="9"/>
-      <c r="E25" s="27" t="s">
+      <c r="E25" s="22" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="27.6">
-      <c r="A26" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B26" s="23" t="s">
+    <row r="26" spans="1:6" ht="27">
+      <c r="A26" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="C26" s="17" t="s">
         <v>53</v>
       </c>
       <c r="D26" s="9"/>
-      <c r="E26" s="27" t="s">
+      <c r="E26" s="22" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="41.4">
-      <c r="A27" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" s="24" t="s">
+    <row r="27" spans="1:6" ht="40.5">
+      <c r="A27" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="C27" s="25" t="s">
+      <c r="C27" s="26" t="s">
         <v>53</v>
       </c>
       <c r="D27" s="9"/>
-      <c r="E27" s="27" t="s">
+      <c r="E27" s="22" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="22" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="27.6">
-      <c r="A29" s="27" t="s">
+    <row r="29" spans="1:6" ht="27">
+      <c r="A29" s="22" t="s">
         <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="41.4">
-      <c r="A30" s="31" t="s">
+    <row r="30" spans="1:6" ht="40.5">
+      <c r="A30" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B30" s="7" t="s">
@@ -1398,15 +1395,15 @@
       <c r="C30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="27" t="s">
+      <c r="E30" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="41.4">
-      <c r="A31" s="31" t="s">
+    <row r="31" spans="1:6" ht="40.5">
+      <c r="A31" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B31" s="7" t="s">
@@ -1415,15 +1412,15 @@
       <c r="C31" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E31" s="27" t="s">
+      <c r="E31" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="27.6">
-      <c r="A32" s="31" t="s">
+    <row r="32" spans="1:6" ht="27">
+      <c r="A32" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B32" s="8" t="s">
@@ -1432,15 +1429,15 @@
       <c r="C32" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E32" s="27" t="s">
+      <c r="E32" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="55.2">
-      <c r="A33" s="31" t="s">
+    <row r="33" spans="1:6" ht="54">
+      <c r="A33" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B33" s="8" t="s">
@@ -1449,15 +1446,15 @@
       <c r="C33" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E33" s="27" t="s">
+      <c r="E33" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="27.6">
-      <c r="A34" s="31" t="s">
+    <row r="34" spans="1:6" ht="27">
+      <c r="A34" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B34" s="9" t="s">
@@ -1469,15 +1466,15 @@
       <c r="D34" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E34" s="27" t="s">
+      <c r="E34" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="27.6">
-      <c r="A35" s="31" t="s">
+    <row r="35" spans="1:6" ht="27">
+      <c r="A35" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B35" s="9" t="s">
@@ -1487,15 +1484,15 @@
         <v>7</v>
       </c>
       <c r="D35" s="9"/>
-      <c r="E35" s="27" t="s">
+      <c r="E35" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="41.4">
-      <c r="A36" s="31" t="s">
+    <row r="36" spans="1:6" ht="40.5">
+      <c r="A36" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B36" s="9" t="s">
@@ -1505,15 +1502,15 @@
         <v>7</v>
       </c>
       <c r="D36" s="9"/>
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="55.2">
-      <c r="A37" s="31" t="s">
+    <row r="37" spans="1:6" ht="54">
+      <c r="A37" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B37" s="9" t="s">
@@ -1523,15 +1520,15 @@
         <v>7</v>
       </c>
       <c r="D37" s="9"/>
-      <c r="E37" s="27" t="s">
+      <c r="E37" s="22" t="s">
         <v>126</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="69">
-      <c r="A38" s="31" t="s">
+    <row r="38" spans="1:6" ht="67.5">
+      <c r="A38" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B38" s="8" t="s">
@@ -1543,12 +1540,12 @@
       <c r="D38" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E38" s="27" t="s">
+      <c r="E38" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="41.4">
-      <c r="A39" s="30" t="s">
+    <row r="39" spans="1:6" ht="40.5">
+      <c r="A39" s="19" t="s">
         <v>22</v>
       </c>
       <c r="B39" s="7" t="s">
@@ -1557,15 +1554,17 @@
       <c r="C39" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D39" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" s="27" t="s">
+      <c r="D39" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E39" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="41.4">
-      <c r="A40" s="30"/>
+    <row r="40" spans="1:6" ht="40.5">
+      <c r="A40" s="19" t="s">
+        <v>22</v>
+      </c>
       <c r="B40" s="7" t="s">
         <v>25</v>
       </c>
@@ -1575,12 +1574,14 @@
       <c r="D40" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E40" s="27" t="s">
+      <c r="E40" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="27.6">
-      <c r="A41" s="30"/>
+    <row r="41" spans="1:6" ht="27">
+      <c r="A41" s="19" t="s">
+        <v>22</v>
+      </c>
       <c r="B41" s="7" t="s">
         <v>27</v>
       </c>
@@ -1590,12 +1591,14 @@
       <c r="D41" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="E41" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="27.6">
-      <c r="A42" s="30"/>
+    <row r="42" spans="1:6" ht="27">
+      <c r="A42" s="19" t="s">
+        <v>22</v>
+      </c>
       <c r="B42" s="8" t="s">
         <v>28</v>
       </c>
@@ -1605,50 +1608,56 @@
       <c r="D42" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E42" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="27.6">
-      <c r="A43" s="30" t="s">
+    <row r="43" spans="1:6" ht="27">
+      <c r="A43" s="19" t="s">
         <v>29</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E43" s="27" t="s">
+      <c r="E43" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="41.4">
-      <c r="A44" s="30"/>
+    <row r="44" spans="1:6" ht="40.5">
+      <c r="A44" s="19" t="s">
+        <v>29</v>
+      </c>
       <c r="B44" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E44" s="27" t="s">
+      <c r="E44" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="27.6">
-      <c r="A45" s="30"/>
+    <row r="45" spans="1:6" ht="27">
+      <c r="A45" s="19" t="s">
+        <v>29</v>
+      </c>
       <c r="B45" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E45" s="27" t="s">
+      <c r="E45" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="27.6">
-      <c r="A46" s="30"/>
+    <row r="46" spans="1:6" ht="27">
+      <c r="A46" s="19" t="s">
+        <v>29</v>
+      </c>
       <c r="B46" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E46" s="27" t="s">
+      <c r="E46" s="22" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="55.2">
-      <c r="A47" s="30" t="s">
+    <row r="47" spans="1:6" ht="40.5">
+      <c r="A47" s="19" t="s">
         <v>34</v>
       </c>
       <c r="B47" s="7" t="s">
@@ -1656,71 +1665,85 @@
       </c>
       <c r="C47" s="7"/>
     </row>
-    <row r="48" spans="1:6" ht="55.2">
-      <c r="A48" s="30"/>
+    <row r="48" spans="1:6" ht="40.5">
+      <c r="A48" s="19" t="s">
+        <v>34</v>
+      </c>
       <c r="B48" s="9" t="s">
         <v>36</v>
       </c>
       <c r="C48" s="9"/>
     </row>
-    <row r="49" spans="1:4" ht="55.2">
-      <c r="A49" s="30"/>
+    <row r="49" spans="1:4" ht="40.5">
+      <c r="A49" s="19" t="s">
+        <v>34</v>
+      </c>
       <c r="B49" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C49" s="9"/>
     </row>
-    <row r="50" spans="1:4" ht="41.4">
-      <c r="A50" s="30" t="s">
+    <row r="50" spans="1:4" ht="40.5">
+      <c r="A50" s="19" t="s">
         <v>38</v>
       </c>
       <c r="B50" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C50" s="12"/>
-    </row>
-    <row r="51" spans="1:4" ht="27.6">
-      <c r="A51" s="30"/>
+      <c r="C50" s="11"/>
+    </row>
+    <row r="51" spans="1:4" ht="27">
+      <c r="A51" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="B51" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C51" s="12"/>
-    </row>
-    <row r="52" spans="1:4" ht="41.4">
-      <c r="A52" s="30"/>
+      <c r="C51" s="11"/>
+    </row>
+    <row r="52" spans="1:4" ht="40.5">
+      <c r="A52" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="B52" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C52" s="12"/>
-    </row>
-    <row r="53" spans="1:4" ht="27.6">
-      <c r="A53" s="30"/>
+      <c r="C52" s="11"/>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="B53" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C53" s="12"/>
-    </row>
-    <row r="54" spans="1:4" ht="27.6">
-      <c r="A54" s="30"/>
+      <c r="C53" s="11"/>
+    </row>
+    <row r="54" spans="1:4" ht="27">
+      <c r="A54" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="B54" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C54" s="9"/>
     </row>
-    <row r="55" spans="1:4" ht="27.6">
-      <c r="A55" s="30"/>
+    <row r="55" spans="1:4" ht="27">
+      <c r="A55" s="19" t="s">
+        <v>38</v>
+      </c>
       <c r="B55" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D55" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="27.6">
-      <c r="A56" s="30" t="s">
+      <c r="D55" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="27">
+      <c r="A56" s="19" t="s">
         <v>45</v>
       </c>
       <c r="B56" s="9" t="s">
@@ -1729,343 +1752,349 @@
       <c r="C56" s="9"/>
     </row>
     <row r="57" spans="1:4">
-      <c r="A57" s="30"/>
+      <c r="A57" s="19" t="s">
+        <v>45</v>
+      </c>
       <c r="B57" s="9" t="s">
         <v>47</v>
       </c>
       <c r="C57" s="9"/>
     </row>
-    <row r="58" spans="1:4" ht="27.6">
-      <c r="A58" s="30"/>
+    <row r="58" spans="1:4">
+      <c r="A58" s="19" t="s">
+        <v>45</v>
+      </c>
       <c r="B58" s="9" t="s">
         <v>48</v>
       </c>
       <c r="C58" s="9"/>
     </row>
-    <row r="59" spans="1:4" ht="27.6">
-      <c r="A59" s="30"/>
+    <row r="59" spans="1:4">
+      <c r="A59" s="19" t="s">
+        <v>45</v>
+      </c>
       <c r="B59" s="9" t="s">
         <v>49</v>
       </c>
       <c r="C59" s="9"/>
     </row>
-    <row r="60" spans="1:4" ht="41.4">
-      <c r="A60" s="22" t="s">
+    <row r="60" spans="1:4" ht="27">
+      <c r="A60" s="19" t="s">
         <v>50</v>
       </c>
       <c r="B60" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C60" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="41.4">
-      <c r="A61" s="22" t="s">
+      <c r="C60" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="40.5">
+      <c r="A61" s="19" t="s">
         <v>50</v>
       </c>
       <c r="B61" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C61" s="11" t="s">
+      <c r="C61" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D61" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="69">
-      <c r="A62" s="22" t="s">
+      <c r="D61" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="54">
+      <c r="A62" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B62" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C62" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D62" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="27.6">
-      <c r="A63" s="22" t="s">
+      <c r="C62" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="27">
+      <c r="A63" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B63" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C63" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D63" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="69">
-      <c r="A64" s="22" t="s">
+      <c r="C63" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D63" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="54">
+      <c r="A64" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B64" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C64" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="69">
-      <c r="A65" s="22" t="s">
+      <c r="C64" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="67.900000000000006">
+      <c r="A65" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B65" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C65" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="41.4">
-      <c r="A66" s="22" t="s">
+      <c r="C65" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="40.5">
+      <c r="A66" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B66" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C66" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66" s="11" t="s">
+      <c r="C66" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="41.4">
-      <c r="A67" s="22" t="s">
+    <row r="67" spans="1:4" ht="40.5">
+      <c r="A67" s="19" t="s">
         <v>54</v>
       </c>
       <c r="B67" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C67" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D67" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="41.4">
-      <c r="A68" s="22" t="s">
+      <c r="C67" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="40.5">
+      <c r="A68" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="B68" s="13" t="s">
+      <c r="B68" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="C68" s="14" t="s">
+      <c r="C68" s="30" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="55.2">
-      <c r="A69" s="22" t="s">
+    <row r="69" spans="1:4" ht="40.5">
+      <c r="A69" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B69" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C69" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D69" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="27.6">
-      <c r="A70" s="22" t="s">
+      <c r="C69" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D69" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="27">
+      <c r="A70" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B70" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C70" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D70" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="69">
-      <c r="A71" s="22" t="s">
+      <c r="C70" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="54">
+      <c r="A71" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B71" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C71" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D71" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="55.2">
-      <c r="A72" s="22" t="s">
+      <c r="C71" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="54">
+      <c r="A72" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B72" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D72" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="82.8">
-      <c r="A73" s="22" t="s">
+      <c r="C72" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="81">
+      <c r="A73" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B73" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C73" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D73" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="41.4">
-      <c r="A74" s="22" t="s">
+      <c r="C73" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="40.5">
+      <c r="A74" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B74" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C74" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="41.4">
-      <c r="A75" s="22" t="s">
+      <c r="C74" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="40.5">
+      <c r="A75" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B75" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C75" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D75" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="41.4">
-      <c r="A76" s="22" t="s">
+      <c r="C75" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="40.5">
+      <c r="A76" s="19" t="s">
         <v>62</v>
       </c>
       <c r="B76" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C76" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D76" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="27.6">
-      <c r="A77" s="22" t="s">
+      <c r="C76" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D76" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="19" t="s">
         <v>70</v>
       </c>
       <c r="B77" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="C77" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D77" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="55.2">
-      <c r="A78" s="22" t="s">
+      <c r="C77" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D77" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="40.5">
+      <c r="A78" s="19" t="s">
         <v>70</v>
       </c>
       <c r="B78" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C78" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D78" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" ht="55.2">
-      <c r="A79" s="22" t="s">
+      <c r="C78" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="54">
+      <c r="A79" s="19" t="s">
         <v>73</v>
       </c>
       <c r="B79" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C79" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" ht="138">
-      <c r="A80" s="22" t="s">
+      <c r="C79" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="121.5">
+      <c r="A80" s="19" t="s">
         <v>73</v>
       </c>
       <c r="B80" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C80" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D80" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="41.4">
-      <c r="A81" s="22" t="s">
+      <c r="C80" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D80" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="27">
+      <c r="A81" s="19" t="s">
         <v>73</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C81" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D81" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="96.6">
-      <c r="A82" s="22" t="s">
+      <c r="C81" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D81" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="94.5">
+      <c r="A82" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B82" s="10" t="s">
+      <c r="B82" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="C82" s="14" t="s">
+      <c r="C82" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="D82" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="55.2">
+      <c r="D82" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="54">
       <c r="A83" s="4" t="s">
         <v>78</v>
       </c>
@@ -2076,148 +2105,141 @@
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="55.2">
-      <c r="A84" s="22" t="s">
+    <row r="84" spans="1:4" ht="54">
+      <c r="A84" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B84" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C84" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D84" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="27.6">
-      <c r="A85" s="22" t="s">
+      <c r="C84" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D84" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="27">
+      <c r="A85" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C85" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D85" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="69">
-      <c r="A86" s="22" t="s">
+      <c r="C85" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D85" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="54">
+      <c r="A86" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B86" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C86" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D86" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="41.4">
-      <c r="A87" s="22" t="s">
+      <c r="C86" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D86" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="40.5">
+      <c r="A87" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B87" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C87" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="D87" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="69">
-      <c r="A88" s="22" t="s">
+      <c r="C87" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D87" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="67.5">
+      <c r="A88" s="19" t="s">
         <v>79</v>
       </c>
       <c r="B88" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C88" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D88" s="11" t="s">
+      <c r="C88" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="372.6">
-      <c r="A89" s="22" t="s">
+    <row r="89" spans="1:4" ht="351">
+      <c r="A89" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B89" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C89" s="11"/>
-    </row>
-    <row r="90" spans="1:4" ht="262.2">
-      <c r="A90" s="22" t="s">
+      <c r="C89" s="10"/>
+    </row>
+    <row r="90" spans="1:4" ht="243">
+      <c r="A90" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B90" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C90" s="11"/>
-    </row>
-    <row r="91" spans="1:4" ht="345">
-      <c r="A91" s="22" t="s">
+      <c r="C90" s="10"/>
+    </row>
+    <row r="91" spans="1:4" ht="310.5">
+      <c r="A91" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B91" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C91" s="11"/>
-    </row>
-    <row r="92" spans="1:4" ht="41.4">
-      <c r="A92" s="22" t="s">
+      <c r="C91" s="10"/>
+    </row>
+    <row r="92" spans="1:4" ht="40.5">
+      <c r="A92" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B92" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C92" s="11"/>
-    </row>
-    <row r="93" spans="1:4" ht="151.80000000000001">
-      <c r="A93" s="22" t="s">
+      <c r="C92" s="10"/>
+    </row>
+    <row r="93" spans="1:4" ht="148.5">
+      <c r="A93" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B93" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="C93" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="276">
-      <c r="A94" s="22" t="s">
+      <c r="C93" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="256.5">
+      <c r="A94" s="19" t="s">
         <v>84</v>
       </c>
       <c r="B94" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="C94" s="11" t="s">
+      <c r="C94" s="10" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A43:A46"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="A56:A59"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000003000000}">
           <x14:formula1>
             <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
@@ -2228,19 +2250,7 @@
           <x14:formula1>
             <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>F14:F22</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A48B76D7-2FF8-47E7-8F2B-2F6199868859}">
-          <x14:formula1>
-            <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>F30:F37</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000001000000}">
-          <x14:formula1>
-            <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C690</xm:sqref>
+          <xm:sqref>F14:F22 C2:C690 F30:F37</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
new adaptation agent - combining expert measures with practical cases
</commit_message>
<xml_diff>
--- a/python/data/Реестр_адапт_мер.xlsx
+++ b/python/data/Реестр_адапт_мер.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nasty\Desktop\climate_measures\python\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB94C3BB-F0FB-4131-88CA-859AAE02DE04}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0702FAC6-A698-4208-A834-3D0A812F74CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="усиление адаптивной способности" sheetId="4" r:id="rId1"/>
+    <sheet name="Мероприятия" sheetId="4" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
+    <externalReference r:id="rId3"/>
   </externalReferences>
   <calcPr calcId="0"/>
 </workbook>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="152">
   <si>
     <t>Адаптационная потребность</t>
   </si>
@@ -465,12 +466,96 @@
   <si>
     <t>Снижение уязвимости</t>
   </si>
+  <si>
+    <t>Сторительство водохранилищ для отвода паводковых вод и последующего использоваия их для орошения/сброс в реки на незатапливаемых участках</t>
+  </si>
+  <si>
+    <t>Использование заливамых участков в качестве сенокосов и пастбищ</t>
+  </si>
+  <si>
+    <t>Использование благоприятной возможности</t>
+  </si>
+  <si>
+    <t>Источник финансирования</t>
+  </si>
+  <si>
+    <t>Средства федерального бюджета</t>
+  </si>
+  <si>
+    <t>Источник</t>
+  </si>
+  <si>
+    <t>Use of insurance loss data by local authorities in Norway. URL: https://climate-adapt.Eea.Europa.Eu/en/metadata/case-studies/use-of-insurance-loss-data-by-local-authorities-in-norway</t>
+  </si>
+  <si>
+    <t>The refurbishment of Gomeznarro park in Madrid focused on storm water retention. URL: https://climate-adapt.Eea.Europa.Eu/en/metadata/case-studies/the-refurbishment-of-gomeznarro-park-in-madrid-focused-on-storm-water-retention</t>
+  </si>
+  <si>
+    <t>Сп 104.13330.2011. URL: https://docs.cntd.ru/document/5200022</t>
+  </si>
+  <si>
+    <t>Санпин 2.1.3684-21. URL: https://docs.cntd.ru/document/573536177</t>
+  </si>
+  <si>
+    <t>Гост р 58330.2–2018. URL: https://docs.cntd.ru/document/1200161976
+Гост р 70523–2022. URL: https://docs.cntd.ru/document/1200194523
+Сто 4.2-5-2015</t>
+  </si>
+  <si>
+    <t>Гост р 70523–2022. URL: https://docs.cntd.ru/document/1200194523</t>
+  </si>
+  <si>
+    <t>Гост р 58330.2–2018. URL: https://docs.cntd.ru/document/1200161976
+Гост р 70523–2022. URL: https://docs.cntd.ru/document/1200194523</t>
+  </si>
+  <si>
+    <t>Гост 16265-89. URL: https://internet-law.ru/gosts/gost/11153/</t>
+  </si>
+  <si>
+    <t>Гост р 58330.2–2018. URL: https://docs.cntd.ru/document/1200161976</t>
+  </si>
+  <si>
+    <t>Гост р 70229-2022. URL: https://docs.cntd.ru/document/1200192285/titles</t>
+  </si>
+  <si>
+    <t>Puglia region's ordinance for outdoor workers
+URL: https://climate-adapt.Eea.Europa.Eu/en/metadata/case-studies/protecting-outdoor-agricultural-workers-from-extreme-heat-in-puglia</t>
+  </si>
+  <si>
+    <t>Государственный реестр селекционных достижений. URL: https://gossortrf.Ru/registry/</t>
+  </si>
+  <si>
+    <t>Гост р 58330.2–2018. URL: https://docs.cntd.ru/document/1200161976
+Сто 4.2-5-2015</t>
+  </si>
+  <si>
+    <t>Гост р 58330.2–2018. URL: https://docs.cntd.ru/document/1200161976
+Гост р 58331.3-2019. URL: https://docs.cntd.ru/document/1200163278
+Гост р 71112–2023. URL: https://docs.cntd.ru/document/1304145400
+Гост 17.1.2.03-90. URL: https://docs.cntd.ru/document/1200012477</t>
+  </si>
+  <si>
+    <t>Гост iso 9261-2016. URL: https://docs.cntd.ru/document/603250219</t>
+  </si>
+  <si>
+    <t>2023 Monitoring Report on the German Strategy for Adaptation to Climate Change. Report by the Interministerial Working Group on Adaptation to Climate Change. – Dessau-Roßlau: German Environment Agency. – 374 p. URL: https://climate-adapt.eea.europa.eu/en/metadata/publications/2023-monitoring-report-on-the-german-strategy-for-adaptation-to-climate-change</t>
+  </si>
+  <si>
+    <t>Рд 52.37.624-2001. URL: https://docs.cntd.ru/document/1200036919</t>
+  </si>
+  <si>
+    <t>Худший пожарный прогноз за последние пять лет. URL: https://earthtouches.me/articles/2025/02/26/hudshij-pozharnyj-prognoz-za-poslednie-pjat-let/</t>
+  </si>
+  <si>
+    <t>Гост р 70568-2022. URL: https://docs.cntd.ru/document/1200194646
+Гост р 70229-2022. URL: https://docs.cntd.ru/document/1200192285/titles</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,8 +594,16 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -523,8 +616,14 @@
         <bgColor theme="7" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -547,11 +646,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top"/>
@@ -642,6 +756,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -668,6 +791,31 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Характеристика МО"/>
+      <sheetName val="снижение уязвимости "/>
+      <sheetName val="снижение подверженности"/>
+      <sheetName val="усиление адаптивной способности"/>
+      <sheetName val="использование благопр возможн"/>
+      <sheetName val="снижение клим рисков для финсис"/>
+      <sheetName val="Данные"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -898,7 +1046,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="30.53125" style="22" bestFit="1" customWidth="1"/>
@@ -907,12 +1055,12 @@
     <col min="4" max="4" width="29.86328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="34.46484375" style="22" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="63.1328125" style="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1328125" style="22"/>
-    <col min="8" max="8" width="9.1328125" style="22" customWidth="1"/>
+    <col min="7" max="7" width="24.3984375" style="22" customWidth="1"/>
+    <col min="8" max="8" width="44.265625" style="22" customWidth="1"/>
     <col min="9" max="16384" width="9.1328125" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="27">
+    <row r="1" spans="1:8" s="3" customFormat="1" ht="27">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -931,8 +1079,14 @@
       <c r="F1" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="27">
+      <c r="G1" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="27">
       <c r="A2" s="12" t="s">
         <v>5</v>
       </c>
@@ -948,8 +1102,11 @@
       <c r="E2" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="27">
+      <c r="G2" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="27">
       <c r="A3" s="12" t="s">
         <v>5</v>
       </c>
@@ -966,7 +1123,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="27">
+    <row r="4" spans="1:8" ht="27">
       <c r="A4" s="12" t="s">
         <v>5</v>
       </c>
@@ -981,7 +1138,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="40.5">
+    <row r="5" spans="1:8" ht="40.5">
       <c r="A5" s="12" t="s">
         <v>5</v>
       </c>
@@ -996,7 +1153,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="67.5">
+    <row r="6" spans="1:8" ht="67.5">
       <c r="A6" s="12" t="s">
         <v>5</v>
       </c>
@@ -1011,7 +1168,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="27">
+    <row r="7" spans="1:8" ht="27">
       <c r="A7" s="12" t="s">
         <v>5</v>
       </c>
@@ -1026,7 +1183,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="40.5">
+    <row r="8" spans="1:8" ht="40.5">
       <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1043,7 +1200,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="54">
+    <row r="9" spans="1:8" ht="54">
       <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
@@ -1059,8 +1216,9 @@
       <c r="E9" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="27">
+      <c r="H9" s="32"/>
+    </row>
+    <row r="10" spans="1:8" ht="27">
       <c r="A10" s="12" t="s">
         <v>5</v>
       </c>
@@ -1076,8 +1234,9 @@
       <c r="E10" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="54">
+      <c r="H10" s="32"/>
+    </row>
+    <row r="11" spans="1:8" ht="57">
       <c r="A11" s="12" t="s">
         <v>5</v>
       </c>
@@ -1091,8 +1250,11 @@
       <c r="E11" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="40.5">
+      <c r="H11" s="33" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="40.5">
       <c r="A12" s="21" t="s">
         <v>62</v>
       </c>
@@ -1106,8 +1268,9 @@
       <c r="E12" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="40.5">
+      <c r="H12" s="33"/>
+    </row>
+    <row r="13" spans="1:8" ht="85.5">
       <c r="A13" s="21" t="s">
         <v>78</v>
       </c>
@@ -1121,8 +1284,11 @@
       <c r="E13" s="22" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="40.5">
+      <c r="H13" s="33" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="40.5">
       <c r="A14" s="12" t="s">
         <v>5</v>
       </c>
@@ -1142,7 +1308,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="27">
+    <row r="15" spans="1:8" ht="27">
       <c r="A15" s="12" t="s">
         <v>5</v>
       </c>
@@ -1162,7 +1328,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="40.5">
+    <row r="16" spans="1:8" ht="40.5">
       <c r="A16" s="12" t="s">
         <v>5</v>
       </c>
@@ -1180,7 +1346,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="54">
+    <row r="17" spans="1:8" ht="54">
       <c r="A17" s="12" t="s">
         <v>5</v>
       </c>
@@ -1198,7 +1364,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="27">
+    <row r="18" spans="1:8" ht="27">
       <c r="A18" s="12" t="s">
         <v>5</v>
       </c>
@@ -1216,7 +1382,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="40.5">
+    <row r="19" spans="1:8" ht="40.5">
       <c r="A19" s="12" t="s">
         <v>5</v>
       </c>
@@ -1234,7 +1400,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="40.5">
+    <row r="20" spans="1:8" ht="40.5">
       <c r="A20" s="12" t="s">
         <v>5</v>
       </c>
@@ -1254,7 +1420,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="40.5">
+    <row r="21" spans="1:8" ht="40.5">
       <c r="A21" s="12" t="s">
         <v>5</v>
       </c>
@@ -1274,7 +1440,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="54">
+    <row r="22" spans="1:8" ht="54">
       <c r="A22" s="12" t="s">
         <v>5</v>
       </c>
@@ -1294,7 +1460,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="27">
+    <row r="23" spans="1:8" ht="27">
       <c r="A23" s="12" t="s">
         <v>5</v>
       </c>
@@ -1309,7 +1475,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:8">
       <c r="A24" s="12" t="s">
         <v>5</v>
       </c>
@@ -1324,7 +1490,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:8">
       <c r="A25" s="12" t="s">
         <v>5</v>
       </c>
@@ -1339,7 +1505,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="27">
+    <row r="26" spans="1:8" ht="27">
       <c r="A26" s="12" t="s">
         <v>5</v>
       </c>
@@ -1354,7 +1520,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="40.5">
+    <row r="27" spans="1:8" ht="40.5">
       <c r="A27" s="12" t="s">
         <v>5</v>
       </c>
@@ -1369,23 +1535,31 @@
         <v>124</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:8">
       <c r="A28" s="22" t="s">
         <v>22</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="27">
+      <c r="E28" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="H28" s="32"/>
+    </row>
+    <row r="29" spans="1:8" ht="27">
       <c r="A29" s="22" t="s">
         <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="40.5">
+      <c r="E29" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="H29" s="32"/>
+    </row>
+    <row r="30" spans="1:8" ht="40.5">
       <c r="A30" s="24" t="s">
         <v>5</v>
       </c>
@@ -1401,8 +1575,14 @@
       <c r="F30" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="40.5">
+      <c r="G30" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="40.5">
       <c r="A31" s="24" t="s">
         <v>5</v>
       </c>
@@ -1418,8 +1598,11 @@
       <c r="F31" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="27">
+      <c r="H31" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="27">
       <c r="A32" s="24" t="s">
         <v>5</v>
       </c>
@@ -1435,8 +1618,11 @@
       <c r="F32" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="54">
+      <c r="H32" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="54">
       <c r="A33" s="24" t="s">
         <v>5</v>
       </c>
@@ -1452,8 +1638,11 @@
       <c r="F33" s="9" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="27">
+      <c r="H33" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="27">
       <c r="A34" s="24" t="s">
         <v>5</v>
       </c>
@@ -1472,8 +1661,9 @@
       <c r="F34" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="27">
+      <c r="H34" s="32"/>
+    </row>
+    <row r="35" spans="1:8" ht="27">
       <c r="A35" s="24" t="s">
         <v>5</v>
       </c>
@@ -1490,8 +1680,9 @@
       <c r="F35" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="40.5">
+      <c r="H35" s="32"/>
+    </row>
+    <row r="36" spans="1:8" ht="40.5">
       <c r="A36" s="24" t="s">
         <v>5</v>
       </c>
@@ -1508,8 +1699,9 @@
       <c r="F36" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="54">
+      <c r="H36" s="32"/>
+    </row>
+    <row r="37" spans="1:8" ht="54">
       <c r="A37" s="24" t="s">
         <v>5</v>
       </c>
@@ -1526,8 +1718,9 @@
       <c r="F37" s="9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="67.5">
+      <c r="H37" s="32"/>
+    </row>
+    <row r="38" spans="1:8" ht="67.5">
       <c r="A38" s="24" t="s">
         <v>5</v>
       </c>
@@ -1543,8 +1736,11 @@
       <c r="E38" s="22" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="40.5">
+      <c r="H38" s="27" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="40.5">
       <c r="A39" s="19" t="s">
         <v>22</v>
       </c>
@@ -1561,7 +1757,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="40.5">
+    <row r="40" spans="1:8" ht="40.5">
       <c r="A40" s="19" t="s">
         <v>22</v>
       </c>
@@ -1578,7 +1774,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="27">
+    <row r="41" spans="1:8" ht="27">
       <c r="A41" s="19" t="s">
         <v>22</v>
       </c>
@@ -1595,7 +1791,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="27">
+    <row r="42" spans="1:8" ht="27">
       <c r="A42" s="19" t="s">
         <v>22</v>
       </c>
@@ -1612,7 +1808,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="27">
+    <row r="43" spans="1:8" ht="27">
       <c r="A43" s="19" t="s">
         <v>29</v>
       </c>
@@ -1623,7 +1819,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="40.5">
+    <row r="44" spans="1:8" ht="40.5">
       <c r="A44" s="19" t="s">
         <v>29</v>
       </c>
@@ -1634,7 +1830,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="27">
+    <row r="45" spans="1:8" ht="27">
       <c r="A45" s="19" t="s">
         <v>29</v>
       </c>
@@ -1645,7 +1841,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="27">
+    <row r="46" spans="1:8" ht="27">
       <c r="A46" s="19" t="s">
         <v>29</v>
       </c>
@@ -1656,7 +1852,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="40.5">
+    <row r="47" spans="1:8" ht="40.5">
       <c r="A47" s="19" t="s">
         <v>34</v>
       </c>
@@ -1664,8 +1860,11 @@
         <v>35</v>
       </c>
       <c r="C47" s="7"/>
-    </row>
-    <row r="48" spans="1:6" ht="40.5">
+      <c r="E47" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="40.5">
       <c r="A48" s="19" t="s">
         <v>34</v>
       </c>
@@ -1673,8 +1872,11 @@
         <v>36</v>
       </c>
       <c r="C48" s="9"/>
-    </row>
-    <row r="49" spans="1:4" ht="40.5">
+      <c r="E48" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="40.5">
       <c r="A49" s="19" t="s">
         <v>34</v>
       </c>
@@ -1682,8 +1884,11 @@
         <v>37</v>
       </c>
       <c r="C49" s="9"/>
-    </row>
-    <row r="50" spans="1:4" ht="40.5">
+      <c r="E49" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="40.5">
       <c r="A50" s="19" t="s">
         <v>38</v>
       </c>
@@ -1691,8 +1896,11 @@
         <v>39</v>
       </c>
       <c r="C50" s="11"/>
-    </row>
-    <row r="51" spans="1:4" ht="27">
+      <c r="E50" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="27">
       <c r="A51" s="19" t="s">
         <v>38</v>
       </c>
@@ -1700,8 +1908,11 @@
         <v>40</v>
       </c>
       <c r="C51" s="11"/>
-    </row>
-    <row r="52" spans="1:4" ht="40.5">
+      <c r="E51" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="40.5">
       <c r="A52" s="19" t="s">
         <v>38</v>
       </c>
@@ -1709,8 +1920,11 @@
         <v>41</v>
       </c>
       <c r="C52" s="11"/>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" s="19" t="s">
         <v>38</v>
       </c>
@@ -1718,8 +1932,11 @@
         <v>42</v>
       </c>
       <c r="C53" s="11"/>
-    </row>
-    <row r="54" spans="1:4" ht="27">
+      <c r="E53" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="27">
       <c r="A54" s="19" t="s">
         <v>38</v>
       </c>
@@ -1727,8 +1944,11 @@
         <v>43</v>
       </c>
       <c r="C54" s="9"/>
-    </row>
-    <row r="55" spans="1:4" ht="27">
+      <c r="E54" s="22" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="94.5">
       <c r="A55" s="19" t="s">
         <v>38</v>
       </c>
@@ -1741,8 +1961,14 @@
       <c r="D55" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" ht="27">
+      <c r="E55" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H55" s="27" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="27">
       <c r="A56" s="19" t="s">
         <v>45</v>
       </c>
@@ -1750,8 +1976,14 @@
         <v>46</v>
       </c>
       <c r="C56" s="9"/>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H56" s="27" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="27">
       <c r="A57" s="19" t="s">
         <v>45</v>
       </c>
@@ -1759,8 +1991,12 @@
         <v>47</v>
       </c>
       <c r="C57" s="9"/>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H57" s="32"/>
+    </row>
+    <row r="58" spans="1:8" ht="27">
       <c r="A58" s="19" t="s">
         <v>45</v>
       </c>
@@ -1768,8 +2004,14 @@
         <v>48</v>
       </c>
       <c r="C58" s="9"/>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H58" s="27" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="27">
       <c r="A59" s="19" t="s">
         <v>45</v>
       </c>
@@ -1777,8 +2019,12 @@
         <v>49</v>
       </c>
       <c r="C59" s="9"/>
-    </row>
-    <row r="60" spans="1:4" ht="27">
+      <c r="E59" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H59" s="32"/>
+    </row>
+    <row r="60" spans="1:8" ht="27">
       <c r="A60" s="19" t="s">
         <v>50</v>
       </c>
@@ -1791,8 +2037,12 @@
       <c r="D60" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" ht="40.5">
+      <c r="E60" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H60" s="32"/>
+    </row>
+    <row r="61" spans="1:8" ht="67.5">
       <c r="A61" s="19" t="s">
         <v>50</v>
       </c>
@@ -1805,8 +2055,14 @@
       <c r="D61" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" ht="54">
+      <c r="E61" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H61" s="27" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="54">
       <c r="A62" s="19" t="s">
         <v>54</v>
       </c>
@@ -1819,8 +2075,14 @@
       <c r="D62" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" ht="27">
+      <c r="E62" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H62" s="27" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="27">
       <c r="A63" s="19" t="s">
         <v>54</v>
       </c>
@@ -1833,8 +2095,12 @@
       <c r="D63" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" ht="54">
+      <c r="E63" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H63" s="32"/>
+    </row>
+    <row r="64" spans="1:8" ht="54">
       <c r="A64" s="19" t="s">
         <v>54</v>
       </c>
@@ -1847,8 +2113,14 @@
       <c r="D64" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" ht="67.900000000000006">
+      <c r="E64" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H64" s="27" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="67.900000000000006">
       <c r="A65" s="19" t="s">
         <v>54</v>
       </c>
@@ -1861,8 +2133,12 @@
       <c r="D65" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" ht="40.5">
+      <c r="E65" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H65" s="32"/>
+    </row>
+    <row r="66" spans="1:8" ht="40.5">
       <c r="A66" s="19" t="s">
         <v>54</v>
       </c>
@@ -1875,8 +2151,14 @@
       <c r="D66" s="10" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" ht="40.5">
+      <c r="E66" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H66" s="27" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="40.5">
       <c r="A67" s="19" t="s">
         <v>54</v>
       </c>
@@ -1889,8 +2171,14 @@
       <c r="D67" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="40.5">
+      <c r="E67" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H67" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="67.5">
       <c r="A68" s="19" t="s">
         <v>54</v>
       </c>
@@ -1900,8 +2188,14 @@
       <c r="C68" s="30" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" ht="40.5">
+      <c r="E68" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H68" s="27" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="40.5">
       <c r="A69" s="19" t="s">
         <v>62</v>
       </c>
@@ -1914,8 +2208,14 @@
       <c r="D69" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" ht="27">
+      <c r="E69" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H69" s="27" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="27">
       <c r="A70" s="19" t="s">
         <v>62</v>
       </c>
@@ -1928,8 +2228,12 @@
       <c r="D70" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" ht="54">
+      <c r="E70" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H70" s="32"/>
+    </row>
+    <row r="71" spans="1:8" ht="54">
       <c r="A71" s="19" t="s">
         <v>62</v>
       </c>
@@ -1942,8 +2246,12 @@
       <c r="D71" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" ht="54">
+      <c r="E71" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H71" s="32"/>
+    </row>
+    <row r="72" spans="1:8" ht="54">
       <c r="A72" s="19" t="s">
         <v>62</v>
       </c>
@@ -1956,8 +2264,12 @@
       <c r="D72" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" ht="81">
+      <c r="E72" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H72" s="32"/>
+    </row>
+    <row r="73" spans="1:8" ht="81">
       <c r="A73" s="19" t="s">
         <v>62</v>
       </c>
@@ -1970,8 +2282,14 @@
       <c r="D73" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" ht="40.5">
+      <c r="E73" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H73" s="27" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="148.5">
       <c r="A74" s="19" t="s">
         <v>62</v>
       </c>
@@ -1984,8 +2302,14 @@
       <c r="D74" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" ht="40.5">
+      <c r="E74" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H74" s="27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="40.5">
       <c r="A75" s="19" t="s">
         <v>62</v>
       </c>
@@ -1998,8 +2322,14 @@
       <c r="D75" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" ht="40.5">
+      <c r="E75" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H75" s="27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="40.5">
       <c r="A76" s="19" t="s">
         <v>62</v>
       </c>
@@ -2012,8 +2342,14 @@
       <c r="D76" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="E76" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H76" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="121.5">
       <c r="A77" s="19" t="s">
         <v>70</v>
       </c>
@@ -2026,8 +2362,14 @@
       <c r="D77" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" ht="40.5">
+      <c r="E77" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H77" s="27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="40.5">
       <c r="A78" s="19" t="s">
         <v>70</v>
       </c>
@@ -2040,8 +2382,14 @@
       <c r="D78" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" ht="54">
+      <c r="E78" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H78" s="27" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="54">
       <c r="A79" s="19" t="s">
         <v>73</v>
       </c>
@@ -2051,8 +2399,15 @@
       <c r="C79" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" ht="121.5">
+      <c r="D79" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E79" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H79" s="32"/>
+    </row>
+    <row r="80" spans="1:8" ht="121.5">
       <c r="A80" s="19" t="s">
         <v>73</v>
       </c>
@@ -2065,8 +2420,14 @@
       <c r="D80" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" ht="27">
+      <c r="E80" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H80" s="33" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" ht="57">
       <c r="A81" s="19" t="s">
         <v>73</v>
       </c>
@@ -2079,8 +2440,14 @@
       <c r="D81" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" ht="94.5">
+      <c r="E81" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H81" s="33" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="94.5">
       <c r="A82" s="19" t="s">
         <v>73</v>
       </c>
@@ -2090,11 +2457,13 @@
       <c r="C82" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="D82" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="54">
+      <c r="D82" s="10"/>
+      <c r="E82" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H82" s="33"/>
+    </row>
+    <row r="83" spans="1:8" ht="54">
       <c r="A83" s="4" t="s">
         <v>78</v>
       </c>
@@ -2104,8 +2473,15 @@
       <c r="C83" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" ht="54">
+      <c r="E83" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="F83" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H83" s="32"/>
+    </row>
+    <row r="84" spans="1:8" ht="54">
       <c r="A84" s="19" t="s">
         <v>79</v>
       </c>
@@ -2118,8 +2494,14 @@
       <c r="D84" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" ht="27">
+      <c r="E84" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H84" s="27" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" ht="27">
       <c r="A85" s="19" t="s">
         <v>79</v>
       </c>
@@ -2132,8 +2514,12 @@
       <c r="D85" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" ht="54">
+      <c r="E85" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H85" s="32"/>
+    </row>
+    <row r="86" spans="1:8" ht="54">
       <c r="A86" s="19" t="s">
         <v>79</v>
       </c>
@@ -2146,8 +2532,12 @@
       <c r="D86" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" ht="40.5">
+      <c r="E86" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H86" s="32"/>
+    </row>
+    <row r="87" spans="1:8" ht="40.5">
       <c r="A87" s="19" t="s">
         <v>79</v>
       </c>
@@ -2160,8 +2550,14 @@
       <c r="D87" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" ht="67.5">
+      <c r="E87" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H87" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="121.5">
       <c r="A88" s="19" t="s">
         <v>79</v>
       </c>
@@ -2174,8 +2570,14 @@
       <c r="D88" s="10" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" ht="351">
+      <c r="E88" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H88" s="27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="351">
       <c r="A89" s="19" t="s">
         <v>84</v>
       </c>
@@ -2183,8 +2585,12 @@
         <v>85</v>
       </c>
       <c r="C89" s="10"/>
-    </row>
-    <row r="90" spans="1:4" ht="243">
+      <c r="E89" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H89" s="32"/>
+    </row>
+    <row r="90" spans="1:8" ht="243">
       <c r="A90" s="19" t="s">
         <v>84</v>
       </c>
@@ -2192,8 +2598,12 @@
         <v>86</v>
       </c>
       <c r="C90" s="10"/>
-    </row>
-    <row r="91" spans="1:4" ht="310.5">
+      <c r="E90" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H90" s="32"/>
+    </row>
+    <row r="91" spans="1:8" ht="310.5">
       <c r="A91" s="19" t="s">
         <v>84</v>
       </c>
@@ -2201,8 +2611,12 @@
         <v>87</v>
       </c>
       <c r="C91" s="10"/>
-    </row>
-    <row r="92" spans="1:4" ht="40.5">
+      <c r="E91" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H91" s="32"/>
+    </row>
+    <row r="92" spans="1:8" ht="121.5">
       <c r="A92" s="19" t="s">
         <v>84</v>
       </c>
@@ -2210,8 +2624,14 @@
         <v>88</v>
       </c>
       <c r="C92" s="10"/>
-    </row>
-    <row r="93" spans="1:4" ht="148.5">
+      <c r="E92" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H92" s="27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" ht="148.5">
       <c r="A93" s="19" t="s">
         <v>84</v>
       </c>
@@ -2221,8 +2641,17 @@
       <c r="C93" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" ht="256.5">
+      <c r="D93" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E93" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H93" s="27" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" ht="256.5">
       <c r="A94" s="19" t="s">
         <v>84</v>
       </c>
@@ -2232,14 +2661,66 @@
       <c r="C94" s="10" t="s">
         <v>21</v>
       </c>
+      <c r="D94" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E94" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H94" s="27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" ht="54">
+      <c r="A95" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B95" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C95" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E95" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="G95" s="31" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" ht="27">
+      <c r="A96" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E96" s="22" t="s">
+        <v>129</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H11" r:id="rId1" display="Https://climate-adapt.Eea.Europa.Eu/en/metadata/case-studies/use-of-insurance-loss-data-by-local-authorities-in-norway" xr:uid="{AAC24D2E-5040-47EE-A963-A2954484439E}"/>
+    <hyperlink ref="H13" r:id="rId2" display="Https://climate-adapt.Eea.Europa.Eu/en/metadata/case-studies/the-refurbishment-of-gomeznarro-park-in-madrid-focused-on-storm-water-retention" xr:uid="{D16E7B38-A838-4C97-A547-1914FD3ABA75}"/>
+    <hyperlink ref="H80" r:id="rId3" display="Https://earthtouches.Me/articles/2025/02/26/hudshij-pozharnyj-prognoz-za-poslednie-pjat-let/?Utm_source=telegram&amp;utm_medium=social&amp;utm_campaign=forest-fire&amp;utm_content=post&amp;utm_term=260225" xr:uid="{65A9E511-4762-43A6-9D00-737B04F61B0A}"/>
+    <hyperlink ref="H81" r:id="rId4" display="Https://earthtouches.Me/articles/2025/02/26/hudshij-pozharnyj-prognoz-za-poslednie-pjat-let/?Utm_source=telegram&amp;utm_medium=social&amp;utm_campaign=forest-fire&amp;utm_content=post&amp;utm_term=260225" xr:uid="{79E2FA45-5AFC-454E-BB01-E0ED5E826B70}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000003000000}">
           <x14:formula1>
             <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
@@ -2250,7 +2731,13 @@
           <x14:formula1>
             <xm:f>'C:\Users\nasty\OneDrive\Рабочий стол\[ответственные за мероприятия.xlsx]Данные'!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>F14:F22 C2:C690 F30:F37</xm:sqref>
+          <xm:sqref>F14:F22 F30:F37 C2:C94 C97:C690</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{67DDAC03-0DAD-4D66-8E01-931EE0D654AB}">
+          <x14:formula1>
+            <xm:f>'C:\Users\nasty\Desktop\climate_measures\python\data\[Реестр_адапт_мер2.xlsx]Данные'!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>F83 G2 G95 G30 C95:C96</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>